<commit_message>
demo: update some forms
</commit_message>
<xml_diff>
--- a/Demo/SCH-STH/demo_sppa_impact_2511_2_child.xlsx
+++ b/Demo/SCH-STH/demo_sppa_impact_2511_2_child.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\SCH-STH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F67D7A11-C1ED-4CF1-B7C3-1E1F93D24F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100A0CB9-EA90-4BE2-82BE-F49557DF0565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -3374,10 +3374,10 @@
       <c r="T33" s="33" t="s">
         <v>453</v>
       </c>
-      <c r="U33" s="72" t="s">
+      <c r="U33" s="33"/>
+      <c r="V33" s="72" t="s">
         <v>76</v>
       </c>
-      <c r="V33" s="17"/>
     </row>
     <row r="34" spans="1:22" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="17"/>

</xml_diff>

<commit_message>
add forms for sch/sth
</commit_message>
<xml_diff>
--- a/Demo/SCH-STH/demo_sppa_impact_2511_2_child.xlsx
+++ b/Demo/SCH-STH/demo_sppa_impact_2511_2_child.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\SCH-STH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100A0CB9-EA90-4BE2-82BE-F49557DF0565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F65B57EB-CD0C-424D-A6AC-EB23CFB79653}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -3371,10 +3371,10 @@
       <c r="Q33" s="17"/>
       <c r="R33" s="17"/>
       <c r="S33" s="17"/>
-      <c r="T33" s="33" t="s">
+      <c r="T33" s="33"/>
+      <c r="U33" s="33" t="s">
         <v>453</v>
       </c>
-      <c r="U33" s="33"/>
       <c r="V33" s="72" t="s">
         <v>76</v>
       </c>

</xml_diff>